<commit_message>
feat: sync sounds, questions, client and server updates
</commit_message>
<xml_diff>
--- a/auction-quiz/server/data/team_pool.xlsx
+++ b/auction-quiz/server/data/team_pool.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -487,89 +487,9 @@
         <v>return 0;</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="str">
-        <v>typedef</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="str">
-        <v>struct</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="str">
-        <v>sizeof()</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="str">
-        <v>pointer*</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="str">
-        <v>while(1)</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="str">
-        <v>break;</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18" t="str">
-        <v>const</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19" t="str">
-        <v>switch()</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20" t="str">
-        <v>case:</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" t="str">
-        <v>void*</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>